<commit_message>
feat(pipeline): update COPQ/FTT data processing, add MCP test fixtures, and deliver September 2026 executive reporting
</commit_message>
<xml_diff>
--- a/Database/CoPQ database 25.xlsx
+++ b/Database/CoPQ database 25.xlsx
@@ -32,8 +32,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May-2026" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jun-2026" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="July-2026" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aug-2026" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep-2026" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep-2026" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aug-2026" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
@@ -15772,7 +15772,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>COPQ Overview (Based on Aug 2026)</t>
+          <t>COPQ Overview (Based on Sep 2026)</t>
         </is>
       </c>
       <c r="B1" s="18" t="n"/>
@@ -15856,13 +15856,13 @@
         </is>
       </c>
       <c r="B3" s="41" t="n">
-        <v>6737.58</v>
+        <v>3095.89</v>
       </c>
       <c r="C3" s="41" t="n">
-        <v>1624.04</v>
+        <v>1229.97</v>
       </c>
       <c r="D3" s="41" t="n">
-        <v>1750.99</v>
+        <v>1574.5</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="43">
@@ -15902,13 +15902,13 @@
         </is>
       </c>
       <c r="B4" s="41" t="n">
-        <v>2179.06</v>
+        <v>2325.06</v>
       </c>
       <c r="C4" s="41" t="n">
-        <v>447.06</v>
+        <v>544.84</v>
       </c>
       <c r="D4" s="41" t="n">
-        <v>237.83</v>
+        <v>125.76</v>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="43">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="41" t="n">
-        <v>101.9</v>
+        <v>97.8</v>
       </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
@@ -15970,9 +15970,11 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>3551.88</v>
-      </c>
-      <c r="C6" s="5" t="n"/>
+        <v>3116.88</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>13.12</v>
+      </c>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -16005,13 +16007,13 @@
         </is>
       </c>
       <c r="B7" s="37" t="n">
-        <v>1298.72</v>
+        <v>1308.72</v>
       </c>
       <c r="C7" s="37" t="n">
-        <v>665.74</v>
+        <v>580.45</v>
       </c>
       <c r="D7" s="37" t="n">
-        <v>4566.61</v>
+        <v>6554.62</v>
       </c>
       <c r="E7" s="37" t="n"/>
       <c r="F7" s="37">
@@ -16045,10 +16047,10 @@
       </c>
       <c r="B8" s="40" t="n"/>
       <c r="C8" s="37" t="n">
-        <v>1595.58</v>
+        <v>1837.15</v>
       </c>
       <c r="D8" s="37" t="n">
-        <v>522.27</v>
+        <v>770.0700000000001</v>
       </c>
       <c r="E8" s="37" t="n"/>
       <c r="F8" s="37">
@@ -16082,7 +16084,7 @@
       </c>
       <c r="B9" s="40" t="n"/>
       <c r="C9" s="37" t="n">
-        <v>493.08</v>
+        <v>513.38</v>
       </c>
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
@@ -16196,7 +16198,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>31.5</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17">
@@ -16211,7 +16213,7 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>279</v>
+        <v>394</v>
       </c>
     </row>
     <row r="18">
@@ -16226,7 +16228,7 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>11</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="19">
@@ -16241,7 +16243,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>84.5</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="20">
@@ -16293,7 +16295,7 @@
         </is>
       </c>
       <c r="B23" s="32" t="n">
-        <v>39553</v>
+        <v>38959</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -16301,7 +16303,7 @@
         </is>
       </c>
       <c r="E23" s="32" t="n">
-        <v>55.5</v>
+        <v>56.5</v>
       </c>
       <c r="F23" s="32" t="n"/>
     </row>
@@ -16312,7 +16314,7 @@
         </is>
       </c>
       <c r="B24" s="32" t="n">
-        <v>44113</v>
+        <v>45571</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -16320,7 +16322,7 @@
         </is>
       </c>
       <c r="E24" s="32" t="n">
-        <v>455</v>
+        <v>524</v>
       </c>
     </row>
     <row r="25">
@@ -16330,7 +16332,7 @@
         </is>
       </c>
       <c r="B25" s="32" t="n">
-        <v>15701</v>
+        <v>13814</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -16338,7 +16340,7 @@
         </is>
       </c>
       <c r="E25" s="32" t="n">
-        <v>112.1</v>
+        <v>95.8</v>
       </c>
     </row>
     <row r="26">
@@ -16348,7 +16350,7 @@
         </is>
       </c>
       <c r="B26" s="32" t="n">
-        <v>8108</v>
+        <v>12610</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -16356,7 +16358,7 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>32.2</v>
+        <v>38.1</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -16371,7 +16373,7 @@
         </is>
       </c>
       <c r="B27" s="32" t="n">
-        <v>11534</v>
+        <v>7801</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -16379,7 +16381,7 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>109.2</v>
+        <v>91.2</v>
       </c>
     </row>
     <row r="28">
@@ -16389,7 +16391,7 @@
         </is>
       </c>
       <c r="B28" s="32" t="n">
-        <v>62242</v>
+        <v>39210</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -16397,7 +16399,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>214.2000000000008</v>
+        <v>123.2000000000001</v>
       </c>
     </row>
     <row r="29">
@@ -16462,7 +16464,7 @@
         </is>
       </c>
       <c r="B33" s="32" t="n">
-        <v>14796</v>
+        <v>9740</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -16470,7 +16472,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34">
@@ -16480,7 +16482,7 @@
         </is>
       </c>
       <c r="B34" s="32" t="n">
-        <v>36945</v>
+        <v>25794</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -16488,7 +16490,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>568.3000000000002</v>
+        <v>498.7</v>
       </c>
     </row>
     <row r="35">
@@ -16498,7 +16500,7 @@
         </is>
       </c>
       <c r="B35" s="32" t="n">
-        <v>17932</v>
+        <v>16934</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -16506,7 +16508,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>204.5</v>
+        <v>191.5</v>
       </c>
     </row>
     <row r="36">
@@ -16516,7 +16518,7 @@
         </is>
       </c>
       <c r="B36" s="32" t="n">
-        <v>120824</v>
+        <v>69184</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -16524,7 +16526,7 @@
         </is>
       </c>
       <c r="E36" s="36" t="n">
-        <v>455</v>
+        <v>368</v>
       </c>
     </row>
     <row r="37">
@@ -16576,7 +16578,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>COPQ Overview (Based on Sep 2026)</t>
+          <t>COPQ Overview (Based on Aug 2026)</t>
         </is>
       </c>
       <c r="B1" s="18" t="n"/>
@@ -16660,13 +16662,11 @@
         </is>
       </c>
       <c r="B3" s="41" t="n">
-        <v>3095.89</v>
-      </c>
-      <c r="C3" s="41" t="n">
-        <v>1229.97</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C3" s="41" t="n"/>
       <c r="D3" s="41" t="n">
-        <v>1574.5</v>
+        <v>80</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="43">
@@ -16705,15 +16705,9 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n">
-        <v>2325.06</v>
-      </c>
-      <c r="C4" s="41" t="n">
-        <v>544.84</v>
-      </c>
-      <c r="D4" s="41" t="n">
-        <v>125.76</v>
-      </c>
+      <c r="B4" s="41" t="n"/>
+      <c r="C4" s="41" t="n"/>
+      <c r="D4" s="41" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="43">
         <f>SUM(B4:E4)</f>
@@ -16738,9 +16732,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="41" t="n">
-        <v>97.8</v>
-      </c>
+      <c r="C5" s="41" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="43">
@@ -16773,12 +16765,8 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B6" s="41" t="n">
-        <v>3333.75</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>13.12</v>
-      </c>
+      <c r="B6" s="41" t="n"/>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -16810,15 +16798,9 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
-        <v>1308.72</v>
-      </c>
-      <c r="C7" s="37" t="n">
-        <v>580.45</v>
-      </c>
-      <c r="D7" s="37" t="n">
-        <v>6554.62</v>
-      </c>
+      <c r="B7" s="37" t="n"/>
+      <c r="C7" s="37" t="n"/>
+      <c r="D7" s="37" t="n"/>
       <c r="E7" s="37" t="n"/>
       <c r="F7" s="37">
         <f>SUM(B7:E7)</f>
@@ -16850,12 +16832,8 @@
         </is>
       </c>
       <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n">
-        <v>1837.15</v>
-      </c>
-      <c r="D8" s="37" t="n">
-        <v>770.0700000000001</v>
-      </c>
+      <c r="C8" s="37" t="n"/>
+      <c r="D8" s="37" t="n"/>
       <c r="E8" s="37" t="n"/>
       <c r="F8" s="37">
         <f>SUM(B8:E8)</f>
@@ -16887,9 +16865,7 @@
         </is>
       </c>
       <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n">
-        <v>513.38</v>
-      </c>
+      <c r="C9" s="37" t="n"/>
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
       <c r="F9" s="37">
@@ -17001,9 +16977,7 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>48</v>
-      </c>
+      <c r="E16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -17016,9 +16990,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n">
-        <v>394</v>
-      </c>
+      <c r="E17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17031,9 +17003,7 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="E18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -17046,9 +17016,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n">
-        <v>75.5</v>
-      </c>
+      <c r="E19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17098,17 +17066,13 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
-        <v>38959</v>
-      </c>
+      <c r="B23" s="32" t="n"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n">
-        <v>56.5</v>
-      </c>
+      <c r="E23" s="32" t="n"/>
       <c r="F23" s="32" t="n"/>
     </row>
     <row r="24">
@@ -17117,17 +17081,13 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
-        <v>45571</v>
-      </c>
+      <c r="B24" s="32" t="n"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n">
-        <v>524</v>
-      </c>
+      <c r="E24" s="32" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17135,17 +17095,13 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n">
-        <v>13814</v>
-      </c>
+      <c r="B25" s="32" t="n"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n">
-        <v>95.8</v>
-      </c>
+      <c r="E25" s="32" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17153,17 +17109,13 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n">
-        <v>12610</v>
-      </c>
+      <c r="B26" s="32" t="n"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>VH3</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n">
-        <v>38.1</v>
-      </c>
+      <c r="E26" s="5" t="n"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>"</t>
@@ -17176,17 +17128,13 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n">
-        <v>7801</v>
-      </c>
+      <c r="B27" s="32" t="n"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>91.2</v>
-      </c>
+      <c r="E27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -17194,17 +17142,13 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
-        <v>39210</v>
-      </c>
+      <c r="B28" s="32" t="n"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n">
-        <v>123.2000000000001</v>
-      </c>
+      <c r="E28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -17267,16 +17211,11 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n">
-        <v>9740</v>
-      </c>
+      <c r="B33" s="32" t="n"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
-      </c>
-      <c r="E33" t="n">
-        <v>129</v>
       </c>
     </row>
     <row r="34">
@@ -17285,16 +17224,11 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n">
-        <v>25794</v>
-      </c>
+      <c r="B34" s="32" t="n"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>VH4</t>
         </is>
-      </c>
-      <c r="E34" t="n">
-        <v>533.4000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -17303,16 +17237,11 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n">
-        <v>16934</v>
-      </c>
+      <c r="B35" s="32" t="n"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
-      </c>
-      <c r="E35" t="n">
-        <v>191.5</v>
       </c>
     </row>
     <row r="36">
@@ -17322,16 +17251,14 @@
         </is>
       </c>
       <c r="B36" s="32" t="n">
-        <v>69184</v>
+        <v>10</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n">
-        <v>368</v>
-      </c>
+      <c r="E36" s="36" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -17382,7 +17309,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>COPQ Overview (Based on Sep 2026)</t>
+          <t>COPQ Overview (Based on Aug 2026)</t>
         </is>
       </c>
       <c r="B1" s="18" t="n"/>
@@ -17466,13 +17393,11 @@
         </is>
       </c>
       <c r="B3" s="41" t="n">
-        <v>3095.89</v>
-      </c>
-      <c r="C3" s="41" t="n">
-        <v>1229.97</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C3" s="41" t="n"/>
       <c r="D3" s="41" t="n">
-        <v>1574.5</v>
+        <v>80</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="43">
@@ -17511,15 +17436,9 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n">
-        <v>2325.06</v>
-      </c>
-      <c r="C4" s="41" t="n">
-        <v>544.84</v>
-      </c>
-      <c r="D4" s="41" t="n">
-        <v>125.76</v>
-      </c>
+      <c r="B4" s="41" t="n"/>
+      <c r="C4" s="41" t="n"/>
+      <c r="D4" s="41" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="43">
         <f>SUM(B4:E4)</f>
@@ -17544,9 +17463,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="41" t="n">
-        <v>97.8</v>
-      </c>
+      <c r="C5" s="41" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="43">
@@ -17579,12 +17496,8 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B6" s="41" t="n">
-        <v>3333.75</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>13.12</v>
-      </c>
+      <c r="B6" s="41" t="n"/>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -17616,15 +17529,9 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
-        <v>1308.72</v>
-      </c>
-      <c r="C7" s="37" t="n">
-        <v>580.45</v>
-      </c>
-      <c r="D7" s="37" t="n">
-        <v>6554.62</v>
-      </c>
+      <c r="B7" s="37" t="n"/>
+      <c r="C7" s="37" t="n"/>
+      <c r="D7" s="37" t="n"/>
       <c r="E7" s="37" t="n"/>
       <c r="F7" s="37">
         <f>SUM(B7:E7)</f>
@@ -17656,12 +17563,8 @@
         </is>
       </c>
       <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n">
-        <v>1837.15</v>
-      </c>
-      <c r="D8" s="37" t="n">
-        <v>770.0700000000001</v>
-      </c>
+      <c r="C8" s="37" t="n"/>
+      <c r="D8" s="37" t="n"/>
       <c r="E8" s="37" t="n"/>
       <c r="F8" s="37">
         <f>SUM(B8:E8)</f>
@@ -17693,9 +17596,7 @@
         </is>
       </c>
       <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n">
-        <v>513.38</v>
-      </c>
+      <c r="C9" s="37" t="n"/>
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
       <c r="F9" s="37">
@@ -17807,9 +17708,7 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>48</v>
-      </c>
+      <c r="E16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -17822,9 +17721,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n">
-        <v>394</v>
-      </c>
+      <c r="E17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17837,9 +17734,7 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="E18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -17852,9 +17747,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n">
-        <v>75.5</v>
-      </c>
+      <c r="E19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17904,17 +17797,13 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
-        <v>38959</v>
-      </c>
+      <c r="B23" s="32" t="n"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n">
-        <v>56.5</v>
-      </c>
+      <c r="E23" s="32" t="n"/>
       <c r="F23" s="32" t="n"/>
     </row>
     <row r="24">
@@ -17923,17 +17812,13 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
-        <v>45571</v>
-      </c>
+      <c r="B24" s="32" t="n"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n">
-        <v>524</v>
-      </c>
+      <c r="E24" s="32" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17941,17 +17826,13 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n">
-        <v>13814</v>
-      </c>
+      <c r="B25" s="32" t="n"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n">
-        <v>95.8</v>
-      </c>
+      <c r="E25" s="32" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17959,17 +17840,13 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n">
-        <v>12610</v>
-      </c>
+      <c r="B26" s="32" t="n"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>VH3</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n">
-        <v>38.1</v>
-      </c>
+      <c r="E26" s="5" t="n"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>"</t>
@@ -17982,17 +17859,13 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n">
-        <v>7801</v>
-      </c>
+      <c r="B27" s="32" t="n"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n">
-        <v>91.2</v>
-      </c>
+      <c r="E27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -18000,17 +17873,13 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
-        <v>39210</v>
-      </c>
+      <c r="B28" s="32" t="n"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n">
-        <v>123.2000000000001</v>
-      </c>
+      <c r="E28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -18073,16 +17942,11 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n">
-        <v>9740</v>
-      </c>
+      <c r="B33" s="32" t="n"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
-      </c>
-      <c r="E33" t="n">
-        <v>129</v>
       </c>
     </row>
     <row r="34">
@@ -18091,16 +17955,11 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n">
-        <v>25794</v>
-      </c>
+      <c r="B34" s="32" t="n"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>VH4</t>
         </is>
-      </c>
-      <c r="E34" t="n">
-        <v>533.4000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -18109,16 +17968,11 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n">
-        <v>16934</v>
-      </c>
+      <c r="B35" s="32" t="n"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
-      </c>
-      <c r="E35" t="n">
-        <v>191.5</v>
       </c>
     </row>
     <row r="36">
@@ -18128,16 +17982,14 @@
         </is>
       </c>
       <c r="B36" s="32" t="n">
-        <v>69184</v>
+        <v>10</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n">
-        <v>368</v>
-      </c>
+      <c r="E36" s="36" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">

</xml_diff>

<commit_message>
fix(database): restore August 2026 data and sandbox test database execution
</commit_message>
<xml_diff>
--- a/Database/CoPQ database 25.xlsx
+++ b/Database/CoPQ database 25.xlsx
@@ -32,8 +32,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="May-2026" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jun-2026" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="July-2026" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep-2026" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aug-2026" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aug-2026" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sep-2026" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
@@ -681,7 +681,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -770,6 +770,16 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15756,12 +15766,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N37"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.1833333333333" customWidth="1" style="20" min="1" max="1"/>
     <col width="15.6333333333333" customWidth="1" style="20" min="2" max="2"/>
     <col width="13.1833333333333" customWidth="1" style="20" min="3" max="3"/>
-    <col width="12.1833333333333" customWidth="1" style="20" min="4" max="6"/>
+    <col width="12.1833333333333" customWidth="1" style="20" min="4" max="4"/>
     <col width="21.725" customWidth="1" style="20" min="7" max="7"/>
     <col width="12.5416666666667" customWidth="1" style="20" min="10" max="10"/>
     <col width="11.5416666666667" customWidth="1" style="20" min="11" max="11"/>
@@ -15772,7 +15782,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>COPQ Overview (Based on Sep 2026)</t>
+          <t>COPQ Overview (Based on Aug 2026)</t>
         </is>
       </c>
       <c r="B1" s="18" t="n"/>
@@ -15856,20 +15866,20 @@
         </is>
       </c>
       <c r="B3" s="41" t="n">
-        <v>3095.89</v>
+        <v>6737.58</v>
       </c>
       <c r="C3" s="41" t="n">
-        <v>1229.97</v>
+        <v>1624.04</v>
       </c>
       <c r="D3" s="41" t="n">
-        <v>1574.5</v>
+        <v>1750.99</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="43">
         <f>SUM(B3:E3)</f>
         <v/>
       </c>
-      <c r="G3" s="38">
+      <c r="G3" s="44">
         <f>B3+C3</f>
         <v/>
       </c>
@@ -15902,20 +15912,20 @@
         </is>
       </c>
       <c r="B4" s="41" t="n">
-        <v>2325.06</v>
+        <v>2179.06</v>
       </c>
       <c r="C4" s="41" t="n">
-        <v>544.84</v>
+        <v>447.06</v>
       </c>
       <c r="D4" s="41" t="n">
-        <v>125.76</v>
+        <v>237.83</v>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="43">
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
-      <c r="G4" s="38">
+      <c r="G4" s="44">
         <f>B4+C4</f>
         <v/>
       </c>
@@ -15935,7 +15945,7 @@
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="41" t="n">
-        <v>97.8</v>
+        <v>101.9</v>
       </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
@@ -15943,7 +15953,7 @@
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
-      <c r="G5" s="38">
+      <c r="G5" s="44">
         <f>B5+C5</f>
         <v/>
       </c>
@@ -15970,18 +15980,16 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>3116.88</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>13.12</v>
-      </c>
+        <v>3551.88</v>
+      </c>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
         <f>SUM(B6:E6)</f>
         <v/>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="44">
         <f>B6+C6</f>
         <v/>
       </c>
@@ -16006,21 +16014,21 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
-        <v>1308.72</v>
-      </c>
-      <c r="C7" s="37" t="n">
-        <v>580.45</v>
-      </c>
-      <c r="D7" s="37" t="n">
-        <v>6554.62</v>
-      </c>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="37">
+      <c r="B7" s="39" t="n">
+        <v>1298.72</v>
+      </c>
+      <c r="C7" s="39" t="n">
+        <v>665.74</v>
+      </c>
+      <c r="D7" s="39" t="n">
+        <v>4566.61</v>
+      </c>
+      <c r="E7" s="39" t="n"/>
+      <c r="F7" s="39">
         <f>SUM(B7:E7)</f>
         <v/>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="44">
         <f>B7+C7</f>
         <v/>
       </c>
@@ -16045,19 +16053,19 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n">
-        <v>1837.15</v>
-      </c>
-      <c r="D8" s="37" t="n">
-        <v>770.0700000000001</v>
-      </c>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="37">
+      <c r="B8" s="45" t="n"/>
+      <c r="C8" s="39" t="n">
+        <v>1595.58</v>
+      </c>
+      <c r="D8" s="39" t="n">
+        <v>522.27</v>
+      </c>
+      <c r="E8" s="39" t="n"/>
+      <c r="F8" s="39">
         <f>SUM(B8:E8)</f>
         <v/>
       </c>
-      <c r="G8" s="38">
+      <c r="G8" s="44">
         <f>B8+C8</f>
         <v/>
       </c>
@@ -16068,7 +16076,7 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="K8" s="37">
+      <c r="K8" s="39">
         <f>K6+K7</f>
         <v/>
       </c>
@@ -16082,24 +16090,24 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n">
-        <v>513.38</v>
-      </c>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="37">
+      <c r="B9" s="45" t="n"/>
+      <c r="C9" s="39" t="n">
+        <v>493.08</v>
+      </c>
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39">
         <f>SUM(B9:E9)</f>
         <v/>
       </c>
-      <c r="G9" s="38">
+      <c r="G9" s="44">
         <f>B9+C9</f>
         <v/>
       </c>
       <c r="H9" s="18" t="n"/>
       <c r="I9" s="18" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="17" t="n"/>
+      <c r="J9" s="46" t="n"/>
+      <c r="K9" s="46" t="n"/>
       <c r="L9" s="18" t="n"/>
       <c r="M9" s="18" t="n"/>
       <c r="N9" s="18" t="n"/>
@@ -16110,34 +16118,34 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="39">
         <f>SUM(B3:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="39">
         <f>SUM(C3:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="39">
         <f>SUM(D3:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="39">
         <f>SUM(E3:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="37">
+      <c r="F10" s="39">
         <f>SUM(B10:E10)</f>
         <v/>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="44">
         <f>B10+C10</f>
         <v/>
       </c>
       <c r="H10" s="18" t="n"/>
       <c r="I10" s="18" t="n"/>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="n"/>
+      <c r="J10" s="46" t="n"/>
+      <c r="K10" s="46" t="n"/>
       <c r="L10" s="18" t="n"/>
       <c r="M10" s="18" t="n"/>
       <c r="N10" s="18" t="n"/>
@@ -16164,6 +16172,7 @@
     <row r="13">
       <c r="L13" s="31" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -16198,7 +16207,7 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>48</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="17">
@@ -16213,7 +16222,7 @@
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>394</v>
+        <v>279</v>
       </c>
     </row>
     <row r="18">
@@ -16228,7 +16237,7 @@
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>6.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19">
@@ -16243,7 +16252,7 @@
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>75.5</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="20">
@@ -16266,6 +16275,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -16294,18 +16304,18 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
-        <v>38959</v>
+      <c r="B23" s="33" t="n">
+        <v>39553</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n">
-        <v>56.5</v>
-      </c>
-      <c r="F23" s="32" t="n"/>
+      <c r="E23" s="33" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="F23" s="33" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -16313,16 +16323,16 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
-        <v>45571</v>
+      <c r="B24" s="33" t="n">
+        <v>44113</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n">
-        <v>524</v>
+      <c r="E24" s="33" t="n">
+        <v>455</v>
       </c>
     </row>
     <row r="25">
@@ -16331,16 +16341,16 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n">
-        <v>13814</v>
+      <c r="B25" s="33" t="n">
+        <v>15701</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n">
-        <v>95.8</v>
+      <c r="E25" s="33" t="n">
+        <v>112.1</v>
       </c>
     </row>
     <row r="26">
@@ -16349,8 +16359,8 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n">
-        <v>12610</v>
+      <c r="B26" s="33" t="n">
+        <v>8108</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -16358,7 +16368,7 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>38.1</v>
+        <v>32.2</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -16372,8 +16382,8 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n">
-        <v>7801</v>
+      <c r="B27" s="33" t="n">
+        <v>11534</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -16381,7 +16391,7 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>91.2</v>
+        <v>109.2</v>
       </c>
     </row>
     <row r="28">
@@ -16390,8 +16400,8 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
-        <v>39210</v>
+      <c r="B28" s="33" t="n">
+        <v>62242</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -16399,7 +16409,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>123.2000000000001</v>
+        <v>214.2000000000008</v>
       </c>
     </row>
     <row r="29">
@@ -16417,11 +16427,12 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="E29" s="36">
+      <c r="E29" s="47">
         <f>SUM(E23:E28)</f>
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -16450,7 +16461,7 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B32" s="32" t="n"/>
+      <c r="B32" s="33" t="n"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>JVB</t>
@@ -16463,8 +16474,8 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n">
-        <v>9740</v>
+      <c r="B33" s="33" t="n">
+        <v>14796</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -16472,7 +16483,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34">
@@ -16481,8 +16492,8 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n">
-        <v>25794</v>
+      <c r="B34" s="33" t="n">
+        <v>36945</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -16490,7 +16501,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>498.7</v>
+        <v>568.3000000000002</v>
       </c>
     </row>
     <row r="35">
@@ -16499,8 +16510,8 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n">
-        <v>16934</v>
+      <c r="B35" s="33" t="n">
+        <v>17932</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -16508,7 +16519,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>191.5</v>
+        <v>204.5</v>
       </c>
     </row>
     <row r="36">
@@ -16517,16 +16528,16 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B36" s="32" t="n">
-        <v>69184</v>
+      <c r="B36" s="33" t="n">
+        <v>120824</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n">
-        <v>368</v>
+      <c r="E36" s="47" t="n">
+        <v>455</v>
       </c>
     </row>
     <row r="37">
@@ -16550,8 +16561,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -16578,7 +16588,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>COPQ Overview (Based on Aug 2026)</t>
+          <t>COPQ Overview (Based on Sep 2026)</t>
         </is>
       </c>
       <c r="B1" s="18" t="n"/>
@@ -16662,11 +16672,13 @@
         </is>
       </c>
       <c r="B3" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="C3" s="41" t="n"/>
+        <v>3095.89</v>
+      </c>
+      <c r="C3" s="41" t="n">
+        <v>1229.97</v>
+      </c>
       <c r="D3" s="41" t="n">
-        <v>80</v>
+        <v>1584.47</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="43">
@@ -16705,9 +16717,15 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n"/>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
+      <c r="B4" s="41" t="n">
+        <v>2325.06</v>
+      </c>
+      <c r="C4" s="41" t="n">
+        <v>544.84</v>
+      </c>
+      <c r="D4" s="41" t="n">
+        <v>125.94</v>
+      </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="43">
         <f>SUM(B4:E4)</f>
@@ -16732,7 +16750,9 @@
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="41" t="n"/>
+      <c r="C5" s="41" t="n">
+        <v>97.8</v>
+      </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="43">
@@ -16765,8 +16785,12 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B6" s="41" t="n"/>
-      <c r="C6" s="5" t="n"/>
+      <c r="B6" s="41" t="n">
+        <v>3116.88</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>13.12</v>
+      </c>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -16798,9 +16822,15 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n"/>
-      <c r="C7" s="37" t="n"/>
-      <c r="D7" s="37" t="n"/>
+      <c r="B7" s="37" t="n">
+        <v>1308.72</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>580.45</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>6558.06</v>
+      </c>
       <c r="E7" s="37" t="n"/>
       <c r="F7" s="37">
         <f>SUM(B7:E7)</f>
@@ -16832,8 +16862,12 @@
         </is>
       </c>
       <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n"/>
-      <c r="D8" s="37" t="n"/>
+      <c r="C8" s="37" t="n">
+        <v>1845.27</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>767.6900000000001</v>
+      </c>
       <c r="E8" s="37" t="n"/>
       <c r="F8" s="37">
         <f>SUM(B8:E8)</f>
@@ -16865,7 +16899,9 @@
         </is>
       </c>
       <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n"/>
+      <c r="C9" s="37" t="n">
+        <v>513.38</v>
+      </c>
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
       <c r="F9" s="37">
@@ -16977,7 +17013,9 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n"/>
+      <c r="E16" s="5" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -16990,7 +17028,9 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n"/>
+      <c r="E17" s="5" t="n">
+        <v>394</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17003,7 +17043,9 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
+      <c r="E18" s="5" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -17016,7 +17058,9 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n"/>
+      <c r="E19" s="5" t="n">
+        <v>75.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17066,13 +17110,17 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n"/>
+      <c r="B23" s="32" t="n">
+        <v>38959</v>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n"/>
+      <c r="E23" s="32" t="n">
+        <v>56.5</v>
+      </c>
       <c r="F23" s="32" t="n"/>
     </row>
     <row r="24">
@@ -17081,13 +17129,17 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n"/>
+      <c r="B24" s="32" t="n">
+        <v>45571</v>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n"/>
+      <c r="E24" s="32" t="n">
+        <v>526</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17095,13 +17147,17 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n"/>
+      <c r="B25" s="32" t="n">
+        <v>13814</v>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n"/>
+      <c r="E25" s="32" t="n">
+        <v>95.8</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17109,13 +17165,17 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n"/>
+      <c r="B26" s="32" t="n">
+        <v>13872</v>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>VH3</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n"/>
+      <c r="E26" s="5" t="n">
+        <v>38.1</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>"</t>
@@ -17128,13 +17188,17 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n"/>
+      <c r="B27" s="32" t="n">
+        <v>7801</v>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n"/>
+      <c r="E27" s="5" t="n">
+        <v>91.2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -17142,13 +17206,17 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n"/>
+      <c r="B28" s="32" t="n">
+        <v>39210</v>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n"/>
+      <c r="E28" s="5" t="n">
+        <v>123.2000000000001</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -17211,11 +17279,16 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n"/>
+      <c r="B33" s="32" t="n">
+        <v>9740</v>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
+      </c>
+      <c r="E33" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="34">
@@ -17224,11 +17297,16 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n"/>
+      <c r="B34" s="32" t="n">
+        <v>25794</v>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>VH4</t>
         </is>
+      </c>
+      <c r="E34" t="n">
+        <v>498.7</v>
       </c>
     </row>
     <row r="35">
@@ -17237,11 +17315,16 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n"/>
+      <c r="B35" s="32" t="n">
+        <v>16934</v>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
+      </c>
+      <c r="E35" t="n">
+        <v>191.5</v>
       </c>
     </row>
     <row r="36">
@@ -17251,14 +17334,16 @@
         </is>
       </c>
       <c r="B36" s="32" t="n">
-        <v>10</v>
+        <v>69184</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n"/>
+      <c r="E36" s="36" t="n">
+        <v>368</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -17309,7 +17394,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>COPQ Overview (Based on Aug 2026)</t>
+          <t>COPQ Overview (Based on Sep 2026)</t>
         </is>
       </c>
       <c r="B1" s="18" t="n"/>
@@ -17393,11 +17478,13 @@
         </is>
       </c>
       <c r="B3" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="C3" s="41" t="n"/>
+        <v>3095.89</v>
+      </c>
+      <c r="C3" s="41" t="n">
+        <v>1229.97</v>
+      </c>
       <c r="D3" s="41" t="n">
-        <v>80</v>
+        <v>1584.47</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="43">
@@ -17436,9 +17523,15 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B4" s="41" t="n"/>
-      <c r="C4" s="41" t="n"/>
-      <c r="D4" s="41" t="n"/>
+      <c r="B4" s="41" t="n">
+        <v>2325.06</v>
+      </c>
+      <c r="C4" s="41" t="n">
+        <v>544.84</v>
+      </c>
+      <c r="D4" s="41" t="n">
+        <v>125.94</v>
+      </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="43">
         <f>SUM(B4:E4)</f>
@@ -17463,7 +17556,9 @@
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="41" t="n"/>
+      <c r="C5" s="41" t="n">
+        <v>97.8</v>
+      </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="43">
@@ -17496,8 +17591,12 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B6" s="41" t="n"/>
-      <c r="C6" s="5" t="n"/>
+      <c r="B6" s="41" t="n">
+        <v>3116.88</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>13.12</v>
+      </c>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -17529,9 +17628,15 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n"/>
-      <c r="C7" s="37" t="n"/>
-      <c r="D7" s="37" t="n"/>
+      <c r="B7" s="37" t="n">
+        <v>1308.72</v>
+      </c>
+      <c r="C7" s="37" t="n">
+        <v>580.45</v>
+      </c>
+      <c r="D7" s="37" t="n">
+        <v>6558.06</v>
+      </c>
       <c r="E7" s="37" t="n"/>
       <c r="F7" s="37">
         <f>SUM(B7:E7)</f>
@@ -17563,8 +17668,12 @@
         </is>
       </c>
       <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n"/>
-      <c r="D8" s="37" t="n"/>
+      <c r="C8" s="37" t="n">
+        <v>1845.27</v>
+      </c>
+      <c r="D8" s="37" t="n">
+        <v>767.6900000000001</v>
+      </c>
       <c r="E8" s="37" t="n"/>
       <c r="F8" s="37">
         <f>SUM(B8:E8)</f>
@@ -17596,7 +17705,9 @@
         </is>
       </c>
       <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n"/>
+      <c r="C9" s="37" t="n">
+        <v>513.38</v>
+      </c>
       <c r="D9" s="37" t="n"/>
       <c r="E9" s="37" t="n"/>
       <c r="F9" s="37">
@@ -17708,7 +17819,9 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n"/>
+      <c r="E16" s="5" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -17721,7 +17834,9 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n"/>
+      <c r="E17" s="5" t="n">
+        <v>394</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17734,7 +17849,9 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
+      <c r="E18" s="5" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -17747,7 +17864,9 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n"/>
+      <c r="E19" s="5" t="n">
+        <v>75.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -17797,13 +17916,17 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n"/>
+      <c r="B23" s="32" t="n">
+        <v>38959</v>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n"/>
+      <c r="E23" s="32" t="n">
+        <v>56.5</v>
+      </c>
       <c r="F23" s="32" t="n"/>
     </row>
     <row r="24">
@@ -17812,13 +17935,17 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n"/>
+      <c r="B24" s="32" t="n">
+        <v>45571</v>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n"/>
+      <c r="E24" s="32" t="n">
+        <v>526</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -17826,13 +17953,17 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n"/>
+      <c r="B25" s="32" t="n">
+        <v>13814</v>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n"/>
+      <c r="E25" s="32" t="n">
+        <v>95.8</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -17840,13 +17971,17 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n"/>
+      <c r="B26" s="32" t="n">
+        <v>13872</v>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>VH3</t>
         </is>
       </c>
-      <c r="E26" s="5" t="n"/>
+      <c r="E26" s="5" t="n">
+        <v>38.1</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
           <t>"</t>
@@ -17859,13 +17994,17 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n"/>
+      <c r="B27" s="32" t="n">
+        <v>7801</v>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
       </c>
-      <c r="E27" s="5" t="n"/>
+      <c r="E27" s="5" t="n">
+        <v>91.2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -17873,13 +18012,17 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n"/>
+      <c r="B28" s="32" t="n">
+        <v>39210</v>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E28" s="5" t="n"/>
+      <c r="E28" s="5" t="n">
+        <v>123.2000000000001</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -17942,11 +18085,16 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n"/>
+      <c r="B33" s="32" t="n">
+        <v>9740</v>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>JV</t>
         </is>
+      </c>
+      <c r="E33" t="n">
+        <v>129</v>
       </c>
     </row>
     <row r="34">
@@ -17955,11 +18103,16 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n"/>
+      <c r="B34" s="32" t="n">
+        <v>25794</v>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>VH4</t>
         </is>
+      </c>
+      <c r="E34" t="n">
+        <v>498.7</v>
       </c>
     </row>
     <row r="35">
@@ -17968,11 +18121,16 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n"/>
+      <c r="B35" s="32" t="n">
+        <v>16934</v>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>VH2</t>
         </is>
+      </c>
+      <c r="E35" t="n">
+        <v>191.5</v>
       </c>
     </row>
     <row r="36">
@@ -17982,14 +18140,16 @@
         </is>
       </c>
       <c r="B36" s="32" t="n">
-        <v>10</v>
+        <v>69184</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n"/>
+      <c r="E36" s="36" t="n">
+        <v>368</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">

</xml_diff>

<commit_message>
fix(database): restore August 2026 trend column in Current month and Sep-26 sheets
</commit_message>
<xml_diff>
--- a/Database/CoPQ database 25.xlsx
+++ b/Database/CoPQ database 25.xlsx
@@ -16172,7 +16172,6 @@
     <row r="13">
       <c r="L13" s="31" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -16275,7 +16274,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
@@ -16432,7 +16430,6 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
@@ -16572,12 +16569,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N37"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.1833333333333" customWidth="1" style="20" min="1" max="1"/>
     <col width="15.6333333333333" customWidth="1" style="20" min="2" max="2"/>
     <col width="13.1833333333333" customWidth="1" style="20" min="3" max="3"/>
-    <col width="12.1833333333333" customWidth="1" style="20" min="4" max="6"/>
+    <col width="12.1833333333333" customWidth="1" style="20" min="4" max="4"/>
     <col width="21.725" customWidth="1" style="20" min="7" max="7"/>
     <col width="12.5416666666667" customWidth="1" style="20" min="10" max="10"/>
     <col width="11.5416666666667" customWidth="1" style="20" min="11" max="11"/>
@@ -16685,7 +16682,7 @@
         <f>SUM(B3:E3)</f>
         <v/>
       </c>
-      <c r="G3" s="38">
+      <c r="G3" s="44">
         <f>B3+C3</f>
         <v/>
       </c>
@@ -16731,7 +16728,7 @@
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
-      <c r="G4" s="38">
+      <c r="G4" s="44">
         <f>B4+C4</f>
         <v/>
       </c>
@@ -16759,7 +16756,7 @@
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
-      <c r="G5" s="38">
+      <c r="G5" s="44">
         <f>B5+C5</f>
         <v/>
       </c>
@@ -16797,7 +16794,7 @@
         <f>SUM(B6:E6)</f>
         <v/>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="44">
         <f>B6+C6</f>
         <v/>
       </c>
@@ -16822,21 +16819,21 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="39" t="n">
         <v>1308.72</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="C7" s="39" t="n">
         <v>580.45</v>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="39" t="n">
         <v>6558.06</v>
       </c>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="37">
+      <c r="E7" s="39" t="n"/>
+      <c r="F7" s="39">
         <f>SUM(B7:E7)</f>
         <v/>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="44">
         <f>B7+C7</f>
         <v/>
       </c>
@@ -16861,19 +16858,19 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n">
+      <c r="B8" s="45" t="n"/>
+      <c r="C8" s="39" t="n">
         <v>1845.27</v>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="39" t="n">
         <v>767.6900000000001</v>
       </c>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="37">
+      <c r="E8" s="39" t="n"/>
+      <c r="F8" s="39">
         <f>SUM(B8:E8)</f>
         <v/>
       </c>
-      <c r="G8" s="38">
+      <c r="G8" s="44">
         <f>B8+C8</f>
         <v/>
       </c>
@@ -16884,7 +16881,7 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="K8" s="37">
+      <c r="K8" s="39">
         <f>K6+K7</f>
         <v/>
       </c>
@@ -16898,24 +16895,24 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n">
+      <c r="B9" s="45" t="n"/>
+      <c r="C9" s="39" t="n">
         <v>513.38</v>
       </c>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="37">
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39">
         <f>SUM(B9:E9)</f>
         <v/>
       </c>
-      <c r="G9" s="38">
+      <c r="G9" s="44">
         <f>B9+C9</f>
         <v/>
       </c>
       <c r="H9" s="18" t="n"/>
       <c r="I9" s="18" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="17" t="n"/>
+      <c r="J9" s="46" t="n"/>
+      <c r="K9" s="46" t="n"/>
       <c r="L9" s="18" t="n"/>
       <c r="M9" s="18" t="n"/>
       <c r="N9" s="18" t="n"/>
@@ -16926,34 +16923,34 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="39">
         <f>SUM(B3:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="39">
         <f>SUM(C3:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="39">
         <f>SUM(D3:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="39">
         <f>SUM(E3:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="37">
+      <c r="F10" s="39">
         <f>SUM(B10:E10)</f>
         <v/>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="44">
         <f>B10+C10</f>
         <v/>
       </c>
       <c r="H10" s="18" t="n"/>
       <c r="I10" s="18" t="n"/>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="n"/>
+      <c r="J10" s="46" t="n"/>
+      <c r="K10" s="46" t="n"/>
       <c r="L10" s="18" t="n"/>
       <c r="M10" s="18" t="n"/>
       <c r="N10" s="18" t="n"/>
@@ -17110,7 +17107,7 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
+      <c r="B23" s="33" t="n">
         <v>38959</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -17118,10 +17115,10 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n">
+      <c r="E23" s="33" t="n">
         <v>56.5</v>
       </c>
-      <c r="F23" s="32" t="n"/>
+      <c r="F23" s="33" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -17129,7 +17126,7 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
+      <c r="B24" s="33" t="n">
         <v>45571</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -17137,7 +17134,7 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n">
+      <c r="E24" s="33" t="n">
         <v>526</v>
       </c>
     </row>
@@ -17147,7 +17144,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n">
+      <c r="B25" s="33" t="n">
         <v>13814</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -17155,7 +17152,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n">
+      <c r="E25" s="33" t="n">
         <v>95.8</v>
       </c>
     </row>
@@ -17165,7 +17162,7 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n">
+      <c r="B26" s="33" t="n">
         <v>13872</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -17188,7 +17185,7 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n">
+      <c r="B27" s="33" t="n">
         <v>7801</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -17206,7 +17203,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
+      <c r="B28" s="33" t="n">
         <v>39210</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -17233,7 +17230,7 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="E29" s="36">
+      <c r="E29" s="47">
         <f>SUM(E23:E28)</f>
         <v/>
       </c>
@@ -17266,7 +17263,7 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B32" s="32" t="n"/>
+      <c r="B32" s="33" t="n"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>JVB</t>
@@ -17279,7 +17276,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n">
+      <c r="B33" s="33" t="n">
         <v>9740</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -17297,7 +17294,7 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n">
+      <c r="B34" s="33" t="n">
         <v>25794</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -17315,7 +17312,7 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n">
+      <c r="B35" s="33" t="n">
         <v>16934</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -17333,7 +17330,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B36" s="32" t="n">
+      <c r="B36" s="33" t="n">
         <v>69184</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -17341,7 +17338,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n">
+      <c r="E36" s="47" t="n">
         <v>368</v>
       </c>
     </row>
@@ -17366,8 +17363,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -17378,12 +17374,12 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N37"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.1833333333333" customWidth="1" style="20" min="1" max="1"/>
     <col width="15.6333333333333" customWidth="1" style="20" min="2" max="2"/>
     <col width="13.1833333333333" customWidth="1" style="20" min="3" max="3"/>
-    <col width="12.1833333333333" customWidth="1" style="20" min="4" max="6"/>
+    <col width="12.1833333333333" customWidth="1" style="20" min="4" max="4"/>
     <col width="21.725" customWidth="1" style="20" min="7" max="7"/>
     <col width="12.5416666666667" customWidth="1" style="20" min="10" max="10"/>
     <col width="11.5416666666667" customWidth="1" style="20" min="11" max="11"/>
@@ -17491,7 +17487,7 @@
         <f>SUM(B3:E3)</f>
         <v/>
       </c>
-      <c r="G3" s="38">
+      <c r="G3" s="44">
         <f>B3+C3</f>
         <v/>
       </c>
@@ -17537,7 +17533,7 @@
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
-      <c r="G4" s="38">
+      <c r="G4" s="44">
         <f>B4+C4</f>
         <v/>
       </c>
@@ -17565,7 +17561,7 @@
         <f>SUM(B5:E5)</f>
         <v/>
       </c>
-      <c r="G5" s="38">
+      <c r="G5" s="44">
         <f>B5+C5</f>
         <v/>
       </c>
@@ -17603,7 +17599,7 @@
         <f>SUM(B6:E6)</f>
         <v/>
       </c>
-      <c r="G6" s="38">
+      <c r="G6" s="44">
         <f>B6+C6</f>
         <v/>
       </c>
@@ -17628,21 +17624,21 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="39" t="n">
         <v>1308.72</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="C7" s="39" t="n">
         <v>580.45</v>
       </c>
-      <c r="D7" s="37" t="n">
+      <c r="D7" s="39" t="n">
         <v>6558.06</v>
       </c>
-      <c r="E7" s="37" t="n"/>
-      <c r="F7" s="37">
+      <c r="E7" s="39" t="n"/>
+      <c r="F7" s="39">
         <f>SUM(B7:E7)</f>
         <v/>
       </c>
-      <c r="G7" s="38">
+      <c r="G7" s="44">
         <f>B7+C7</f>
         <v/>
       </c>
@@ -17667,19 +17663,19 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n"/>
-      <c r="C8" s="37" t="n">
+      <c r="B8" s="45" t="n"/>
+      <c r="C8" s="39" t="n">
         <v>1845.27</v>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="39" t="n">
         <v>767.6900000000001</v>
       </c>
-      <c r="E8" s="37" t="n"/>
-      <c r="F8" s="37">
+      <c r="E8" s="39" t="n"/>
+      <c r="F8" s="39">
         <f>SUM(B8:E8)</f>
         <v/>
       </c>
-      <c r="G8" s="38">
+      <c r="G8" s="44">
         <f>B8+C8</f>
         <v/>
       </c>
@@ -17690,7 +17686,7 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="K8" s="37">
+      <c r="K8" s="39">
         <f>K6+K7</f>
         <v/>
       </c>
@@ -17704,24 +17700,24 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n"/>
-      <c r="C9" s="37" t="n">
+      <c r="B9" s="45" t="n"/>
+      <c r="C9" s="39" t="n">
         <v>513.38</v>
       </c>
-      <c r="D9" s="37" t="n"/>
-      <c r="E9" s="37" t="n"/>
-      <c r="F9" s="37">
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39">
         <f>SUM(B9:E9)</f>
         <v/>
       </c>
-      <c r="G9" s="38">
+      <c r="G9" s="44">
         <f>B9+C9</f>
         <v/>
       </c>
       <c r="H9" s="18" t="n"/>
       <c r="I9" s="18" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="17" t="n"/>
+      <c r="J9" s="46" t="n"/>
+      <c r="K9" s="46" t="n"/>
       <c r="L9" s="18" t="n"/>
       <c r="M9" s="18" t="n"/>
       <c r="N9" s="18" t="n"/>
@@ -17732,34 +17728,34 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="B10" s="37">
+      <c r="B10" s="39">
         <f>SUM(B3:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="39">
         <f>SUM(C3:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="37">
+      <c r="D10" s="39">
         <f>SUM(D3:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="39">
         <f>SUM(E3:E9)</f>
         <v/>
       </c>
-      <c r="F10" s="37">
+      <c r="F10" s="39">
         <f>SUM(B10:E10)</f>
         <v/>
       </c>
-      <c r="G10" s="38">
+      <c r="G10" s="44">
         <f>B10+C10</f>
         <v/>
       </c>
       <c r="H10" s="18" t="n"/>
       <c r="I10" s="18" t="n"/>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="n"/>
+      <c r="J10" s="46" t="n"/>
+      <c r="K10" s="46" t="n"/>
       <c r="L10" s="18" t="n"/>
       <c r="M10" s="18" t="n"/>
       <c r="N10" s="18" t="n"/>
@@ -17916,7 +17912,7 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
+      <c r="B23" s="33" t="n">
         <v>38959</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -17924,10 +17920,10 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="E23" s="32" t="n">
+      <c r="E23" s="33" t="n">
         <v>56.5</v>
       </c>
-      <c r="F23" s="32" t="n"/>
+      <c r="F23" s="33" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -17935,7 +17931,7 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="B24" s="32" t="n">
+      <c r="B24" s="33" t="n">
         <v>45571</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -17943,7 +17939,7 @@
           <t>JV2</t>
         </is>
       </c>
-      <c r="E24" s="32" t="n">
+      <c r="E24" s="33" t="n">
         <v>526</v>
       </c>
     </row>
@@ -17953,7 +17949,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B25" s="32" t="n">
+      <c r="B25" s="33" t="n">
         <v>13814</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -17961,7 +17957,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="E25" s="32" t="n">
+      <c r="E25" s="33" t="n">
         <v>95.8</v>
       </c>
     </row>
@@ -17971,7 +17967,7 @@
           <t>VH3</t>
         </is>
       </c>
-      <c r="B26" s="32" t="n">
+      <c r="B26" s="33" t="n">
         <v>13872</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -17994,7 +17990,7 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B27" s="32" t="n">
+      <c r="B27" s="33" t="n">
         <v>7801</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -18012,7 +18008,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
+      <c r="B28" s="33" t="n">
         <v>39210</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -18039,7 +18035,7 @@
           <t>CLG</t>
         </is>
       </c>
-      <c r="E29" s="36">
+      <c r="E29" s="47">
         <f>SUM(E23:E28)</f>
         <v/>
       </c>
@@ -18072,7 +18068,7 @@
           <t>JVB</t>
         </is>
       </c>
-      <c r="B32" s="32" t="n"/>
+      <c r="B32" s="33" t="n"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>JVB</t>
@@ -18085,7 +18081,7 @@
           <t>JV</t>
         </is>
       </c>
-      <c r="B33" s="32" t="n">
+      <c r="B33" s="33" t="n">
         <v>9740</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -18103,7 +18099,7 @@
           <t>VH4</t>
         </is>
       </c>
-      <c r="B34" s="32" t="n">
+      <c r="B34" s="33" t="n">
         <v>25794</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -18121,7 +18117,7 @@
           <t>VH2</t>
         </is>
       </c>
-      <c r="B35" s="32" t="n">
+      <c r="B35" s="33" t="n">
         <v>16934</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -18139,7 +18135,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="B36" s="32" t="n">
+      <c r="B36" s="33" t="n">
         <v>69184</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -18147,7 +18143,7 @@
           <t>VH</t>
         </is>
       </c>
-      <c r="E36" s="36" t="n">
+      <c r="E36" s="47" t="n">
         <v>368</v>
       </c>
     </row>
@@ -18172,8 +18168,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix(ftt): sort top 3 defects by quantity desc with max rate ordering for stacked chart and clean gitignore
</commit_message>
<xml_diff>
--- a/Database/CoPQ database 25.xlsx
+++ b/Database/CoPQ database 25.xlsx
@@ -16783,11 +16783,9 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>3116.88</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>13.12</v>
-      </c>
+        <v>3130</v>
+      </c>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -17212,7 +17210,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>123.2000000000001</v>
+        <v>123.2</v>
       </c>
     </row>
     <row r="29">
@@ -17295,7 +17293,7 @@
         </is>
       </c>
       <c r="B34" s="33" t="n">
-        <v>25794</v>
+        <v>25919</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -17303,7 +17301,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>498.7</v>
+        <v>500.8</v>
       </c>
     </row>
     <row r="35">
@@ -17588,11 +17586,9 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>3116.88</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>13.12</v>
-      </c>
+        <v>3130</v>
+      </c>
+      <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="43">
@@ -18017,7 +18013,7 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>123.2000000000001</v>
+        <v>123.2</v>
       </c>
     </row>
     <row r="29">
@@ -18100,7 +18096,7 @@
         </is>
       </c>
       <c r="B34" s="33" t="n">
-        <v>25794</v>
+        <v>25919</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -18108,7 +18104,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>498.7</v>
+        <v>500.8</v>
       </c>
     </row>
     <row r="35">

</xml_diff>